<commit_message>
Add book covers build scripts and update promotion files
</commit_message>
<xml_diff>
--- a/Others/Promotion/Channels.xlsx
+++ b/Others/Promotion/Channels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kapil\Books\Others\Promotion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B12AAA-6890-4BA1-8285-7B6403C7584D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CA94B7-B1D7-47C5-BB2A-D447639922B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C80F0329-09F5-452E-B960-17D634B62AEB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="40">
   <si>
     <t>Facebook</t>
   </si>
@@ -144,6 +144,21 @@
   </si>
   <si>
     <t>PSYCHOLOGICAL THRILLERS</t>
+  </si>
+  <si>
+    <t>Twochanins 29Jun</t>
+  </si>
+  <si>
+    <t>Other Mothers on 29Jun</t>
+  </si>
+  <si>
+    <t>Fourth Step 28Jun</t>
+  </si>
+  <si>
+    <t>Thriller, Mystery, &amp; Psychological Suspense Book Recommendations!</t>
+  </si>
+  <si>
+    <t>TwoChains 29Jun</t>
   </si>
 </sst>
 </file>
@@ -197,11 +212,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{868B402B-A569-4BD1-827F-67F1FC187D65}">
-  <dimension ref="C4:K17"/>
+  <dimension ref="C4:K18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="30.85546875" bestFit="1" customWidth="1"/>
@@ -749,9 +765,9 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>2100</v>
-      </c>
-      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H13" t="s">
@@ -761,7 +777,7 @@
         <v>11</v>
       </c>
       <c r="K13" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="3:11" x14ac:dyDescent="0.25">
@@ -791,20 +807,26 @@
       </c>
     </row>
     <row r="15" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" t="s">
+        <v>15</v>
+      </c>
+      <c r="K15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
         <v>18</v>
       </c>
-      <c r="D15" t="s">
-        <v>0</v>
-      </c>
-      <c r="E15" t="s">
-        <v>1</v>
-      </c>
-      <c r="G15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>0</v>
       </c>
@@ -821,7 +843,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
         <v>0</v>
       </c>
@@ -839,6 +861,23 @@
       </c>
       <c r="I17" t="s">
         <v>11</v>
+      </c>
+      <c r="K17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <v>25</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K18" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>